<commit_message>
Nuevos cambios en los archivos, es todo.
</commit_message>
<xml_diff>
--- a/Entregables/CurvaS.xlsx
+++ b/Entregables/CurvaS.xlsx
@@ -1,30 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30431"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emanuel\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2CC8254-9038-42B5-90C4-3C0B98FCB70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
   <si>
     <t>Meses</t>
   </si>
@@ -45,13 +57,19 @@
   </si>
   <si>
     <t>Noviembre</t>
+  </si>
+  <si>
+    <t>Curva S</t>
+  </si>
+  <si>
+    <t>Proyectada</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,59 +394,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1">
         <v>1</v>
       </c>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9">
       <c r="A2" s="1">
         <v>0.95</v>
       </c>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
       <c r="A3" s="1">
         <v>0.85</v>
       </c>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
       <c r="A4" s="1">
         <v>0.7</v>
       </c>
       <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" s="1">
         <v>0.35</v>
       </c>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="A6" s="1">
         <v>0.15</v>
       </c>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="A7" s="1">
         <v>0.05</v>
       </c>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9">
       <c r="A8" s="1">
         <v>0</v>
       </c>
       <c r="B8" s="3"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9">
       <c r="B9" t="s">
         <v>0</v>
       </c>
@@ -451,6 +470,88 @@
         <v>5</v>
       </c>
       <c r="I9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="1">
+        <v>1</v>
+      </c>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="1">
+        <v>0.95</v>
+      </c>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="1">
+        <v>0.85</v>
+      </c>
+      <c r="G15" s="3"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="1">
+        <v>0.35</v>
+      </c>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="C19" s="3"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="1">
+        <v>0</v>
+      </c>
+      <c r="B20" s="3"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="B21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" t="s">
+        <v>2</v>
+      </c>
+      <c r="F21" t="s">
+        <v>3</v>
+      </c>
+      <c r="G21" t="s">
+        <v>4</v>
+      </c>
+      <c r="H21" t="s">
+        <v>5</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Preparando backend para Render
</commit_message>
<xml_diff>
--- a/Entregables/CurvaS.xlsx
+++ b/Entregables/CurvaS.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30431"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emanuel\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\M\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2CC8254-9038-42B5-90C4-3C0B98FCB70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
   <si>
     <t>Meses</t>
   </si>
@@ -63,13 +62,16 @@
   </si>
   <si>
     <t>Proyectada</t>
+  </si>
+  <si>
+    <t>Julio</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,60 +396,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1">
         <v>1</v>
       </c>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0.95</v>
       </c>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>0.85</v>
       </c>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>0.7</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>0.35</v>
       </c>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>0.15</v>
       </c>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>0.05</v>
       </c>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>0</v>
       </c>
       <c r="B8" s="3"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>0</v>
       </c>
@@ -458,7 +460,7 @@
         <v>2</v>
       </c>
       <c r="E9" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F9" t="s">
         <v>3</v>
@@ -473,7 +475,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
         <v>7</v>
       </c>
@@ -481,55 +483,55 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>1</v>
       </c>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>0.95</v>
       </c>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>0.85</v>
       </c>
       <c r="G15" s="3"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>0.7</v>
       </c>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>0.35</v>
       </c>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>0.15</v>
       </c>
       <c r="D18" s="3"/>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>0.05</v>
       </c>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>0</v>
       </c>
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>0</v>
       </c>

</xml_diff>